<commit_message>
0.8.0: network appliance recognition; 02-vs-04 conflict kinds and levels; 04 notes 02 recommendations
</commit_message>
<xml_diff>
--- a/examples/sample-output/Contoso_Azure巡检报告_2026年10月/03_可靠性与安全巡检问题清单.xlsx
+++ b/examples/sample-output/Contoso_Azure巡检报告_2026年10月/03_可靠性与安全巡检问题清单.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30625"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wez\AppData\Local\Temp\azinspect-sample-9n18lti6\2026-09\reports\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wez\AppData\Local\Temp\azinspect-sample-f6nzzhop\2026-09\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{608E9228-ACFF-4F4A-8C58-0EE5885A3306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA6D4001-3FB6-4A91-86D4-4B49FB6F9576}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2280" yWindow="2280" windowWidth="16920" windowHeight="10450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="概览" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">上月问题处理情况!$A$3:$G$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">检查覆盖!$A$3:$F$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">概览!$A$3:$H$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">问题清单!$A$3:$W$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">问题清单!$A$3:$W$28</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="720" uniqueCount="352">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="733" uniqueCount="360">
   <si>
     <t>示例客户 可靠性与安全巡检问题清单（2026年10月26日只读读取）</t>
   </si>
@@ -316,6 +316,9 @@
     <t>S-I8</t>
   </si>
   <si>
+    <t>1 台虚拟机</t>
+  </si>
+  <si>
     <t>Key Vault</t>
   </si>
   <si>
@@ -731,6 +734,27 @@
   </si>
   <si>
     <t>来宾账号 1；来宾账号 2</t>
+  </si>
+  <si>
+    <t>S-I8-c51a20</t>
+  </si>
+  <si>
+    <t>shop-net-rg</t>
+  </si>
+  <si>
+    <t>1 台网络设备</t>
+  </si>
+  <si>
+    <t>订阅 shop-prod 有 1 台网络设备（edge-fw-01）允许管理员用密码登录，其中 1 台绑定了公网 IP。网络设备的管理员通常使用密码，关闭密码登录不适用，重点是限制管理口的访问。按当前 NSG，edge-fw-01 的 22 端口没有对公网开放，风险在于以后放开端口或从内网横向登录。</t>
+  </si>
+  <si>
+    <t>管理口（SSH、HTTPS）只允许受信地址访问、不对公网开放（用 NSG 或设备自身的可信主机设置），管理员账号启用多因素认证并定期更换密码；按厂商建议及时升级设备系统。</t>
+  </si>
+  <si>
+    <t>虚拟机定期做补丁评估，公网可达的 Linux 禁用密码登录</t>
+  </si>
+  <si>
+    <t>edge-fw-01</t>
   </si>
   <si>
     <t>S-I11-0022c1</t>
@@ -1365,7 +1389,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-895D-4E72-869D-B03AEFAA37B5}"/>
+              <c16:uniqueId val="{00000000-4F47-4CA9-A992-2787A1D6BA9D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1505,7 +1529,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-895D-4E72-869D-B03AEFAA37B5}"/>
+              <c16:uniqueId val="{00000001-4F47-4CA9-A992-2787A1D6BA9D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1645,7 +1669,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-895D-4E72-869D-B03AEFAA37B5}"/>
+              <c16:uniqueId val="{00000002-4F47-4CA9-A992-2787A1D6BA9D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1893,7 +1917,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-4000-4AEF-83C1-059E77E68EDB}"/>
+              <c16:uniqueId val="{00000000-DD58-40AA-9C3A-809B7157C8DF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2032,7 +2056,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="16">
                   <c:v>0</c:v>
@@ -2063,7 +2087,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-4000-4AEF-83C1-059E77E68EDB}"/>
+              <c16:uniqueId val="{00000001-DD58-40AA-9C3A-809B7157C8DF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2233,7 +2257,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-4000-4AEF-83C1-059E77E68EDB}"/>
+              <c16:uniqueId val="{00000002-DD58-40AA-9C3A-809B7157C8DF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3515,17 +3539,17 @@
         <v>0</v>
       </c>
       <c r="E33" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F33" s="1">
         <v>0</v>
       </c>
       <c r="G33" s="1">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>13</v>
+        <v>90</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.35">
@@ -3533,10 +3557,10 @@
         <v>49</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D34" s="1">
         <v>0</v>
@@ -3552,7 +3576,7 @@
         <v>1</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.35">
@@ -3560,10 +3584,10 @@
         <v>49</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D35" s="1">
         <v>0</v>
@@ -3587,10 +3611,10 @@
         <v>49</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D36" s="1">
         <v>0</v>
@@ -3606,7 +3630,7 @@
         <v>1</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.35">
@@ -3621,7 +3645,7 @@
       </c>
       <c r="E37" s="1">
         <f>SUM(E4:E36)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F37" s="1">
         <f>SUM(F4:F36)</f>
@@ -3629,7 +3653,7 @@
       </c>
       <c r="G37" s="1">
         <f>SUM(G4:G36)</f>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H37" s="1"/>
     </row>
@@ -3646,7 +3670,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:W27"/>
+  <dimension ref="A1:W28"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="6" width="16" customWidth="1"/>
@@ -3664,7 +3688,7 @@
   <sheetData>
     <row r="1" spans="1:23" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -3691,7 +3715,7 @@
     </row>
     <row r="2" spans="1:23" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -3727,69 +3751,69 @@
         <v>3</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Q3" s="2" t="s">
         <v>9</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="S3" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="T3" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="U3" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="V3" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="W3" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:23" ht="100" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>10</v>
@@ -3801,49 +3825,49 @@
         <v>5</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H4" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="P4" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="Q4" s="1">
+        <v>1</v>
+      </c>
+      <c r="R4" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="I4" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="N4" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="O4" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="P4" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="Q4" s="1">
-        <v>1</v>
-      </c>
-      <c r="R4" s="1" t="s">
-        <v>122</v>
-      </c>
       <c r="S4" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="T4" s="1"/>
       <c r="U4" s="1"/>
@@ -3852,7 +3876,7 @@
     </row>
     <row r="5" spans="1:23" ht="25" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>10</v>
@@ -3864,28 +3888,28 @@
         <v>5</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="M5" s="1"/>
       <c r="N5" s="1"/>
@@ -3895,10 +3919,10 @@
         <v>1</v>
       </c>
       <c r="R5" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="S5" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="T5" s="1"/>
       <c r="U5" s="1"/>
@@ -3907,7 +3931,7 @@
     </row>
     <row r="6" spans="1:23" ht="100" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>10</v>
@@ -3919,47 +3943,47 @@
         <v>5</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="M6" s="1"/>
       <c r="N6" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="Q6" s="1">
         <v>1</v>
       </c>
       <c r="R6" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="S6" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="T6" s="1"/>
       <c r="U6" s="1"/>
@@ -3968,7 +3992,7 @@
     </row>
     <row r="7" spans="1:23" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>10</v>
@@ -3980,28 +4004,28 @@
         <v>5</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="M7" s="1"/>
       <c r="N7" s="1"/>
@@ -4011,10 +4035,10 @@
         <v>1</v>
       </c>
       <c r="R7" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="S7" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="T7" s="1"/>
       <c r="U7" s="1"/>
@@ -4023,7 +4047,7 @@
     </row>
     <row r="8" spans="1:23" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>49</v>
@@ -4035,28 +4059,28 @@
         <v>5</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="M8" s="1"/>
       <c r="N8" s="1"/>
@@ -4066,10 +4090,10 @@
         <v>1</v>
       </c>
       <c r="R8" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="S8" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="T8" s="1"/>
       <c r="U8" s="1"/>
@@ -4078,7 +4102,7 @@
     </row>
     <row r="9" spans="1:23" ht="100" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>49</v>
@@ -4090,47 +4114,47 @@
         <v>5</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="M9" s="1"/>
       <c r="N9" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="Q9" s="1">
         <v>1</v>
       </c>
       <c r="R9" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="S9" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="T9" s="1"/>
       <c r="U9" s="1"/>
@@ -4139,7 +4163,7 @@
     </row>
     <row r="10" spans="1:23" ht="50" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>49</v>
@@ -4151,49 +4175,49 @@
         <v>5</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H10" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="N10" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="O10" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="P10" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="Q10" s="1">
+        <v>1</v>
+      </c>
+      <c r="R10" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="I10" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="K10" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="L10" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="M10" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="N10" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="O10" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="P10" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="Q10" s="1">
-        <v>1</v>
-      </c>
-      <c r="R10" s="1" t="s">
-        <v>166</v>
-      </c>
       <c r="S10" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="T10" s="1"/>
       <c r="U10" s="1"/>
@@ -4202,7 +4226,7 @@
     </row>
     <row r="11" spans="1:23" ht="25" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>10</v>
@@ -4214,7 +4238,7 @@
         <v>6</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F11" s="1"/>
       <c r="G11" s="1" t="s">
@@ -4222,16 +4246,16 @@
       </c>
       <c r="H11" s="1"/>
       <c r="I11" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="M11" s="1"/>
       <c r="N11" s="1"/>
@@ -4241,10 +4265,10 @@
         <v>4</v>
       </c>
       <c r="R11" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="S11" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="T11" s="1"/>
       <c r="U11" s="1"/>
@@ -4253,7 +4277,7 @@
     </row>
     <row r="12" spans="1:23" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>10</v>
@@ -4265,28 +4289,28 @@
         <v>6</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="M12" s="1"/>
       <c r="N12" s="1"/>
@@ -4296,10 +4320,10 @@
         <v>1</v>
       </c>
       <c r="R12" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="S12" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="T12" s="1"/>
       <c r="U12" s="1"/>
@@ -4308,7 +4332,7 @@
     </row>
     <row r="13" spans="1:23" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>10</v>
@@ -4320,47 +4344,47 @@
         <v>6</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="M13" s="1"/>
       <c r="N13" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="O13" s="1" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="P13" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="Q13" s="1">
         <v>1</v>
       </c>
       <c r="R13" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="S13" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="T13" s="1"/>
       <c r="U13" s="1"/>
@@ -4369,7 +4393,7 @@
     </row>
     <row r="14" spans="1:23" ht="50" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>10</v>
@@ -4381,47 +4405,47 @@
         <v>6</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="M14" s="1"/>
       <c r="N14" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="O14" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="P14" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="Q14" s="1">
         <v>1</v>
       </c>
       <c r="R14" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="S14" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="T14" s="1"/>
       <c r="U14" s="1"/>
@@ -4430,7 +4454,7 @@
     </row>
     <row r="15" spans="1:23" ht="25" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>10</v>
@@ -4442,7 +4466,7 @@
         <v>6</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F15" s="1"/>
       <c r="G15" s="1" t="s">
@@ -4450,16 +4474,16 @@
       </c>
       <c r="H15" s="1"/>
       <c r="I15" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="M15" s="1"/>
       <c r="N15" s="1"/>
@@ -4469,10 +4493,10 @@
         <v>2</v>
       </c>
       <c r="R15" s="1" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="S15" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="T15" s="1"/>
       <c r="U15" s="1"/>
@@ -4481,7 +4505,7 @@
     </row>
     <row r="16" spans="1:23" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>10</v>
@@ -4493,26 +4517,26 @@
         <v>6</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F16" s="1"/>
       <c r="G16" s="1" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="L16" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="M16" s="1"/>
       <c r="N16" s="1"/>
@@ -4522,10 +4546,10 @@
         <v>1</v>
       </c>
       <c r="R16" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S16" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="T16" s="1"/>
       <c r="U16" s="1"/>
@@ -4534,7 +4558,7 @@
     </row>
     <row r="17" spans="1:23" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>10</v>
@@ -4546,28 +4570,28 @@
         <v>6</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="M17" s="1"/>
       <c r="N17" s="1"/>
@@ -4577,10 +4601,10 @@
         <v>1</v>
       </c>
       <c r="R17" s="1" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="S17" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="T17" s="1"/>
       <c r="U17" s="1"/>
@@ -4589,7 +4613,7 @@
     </row>
     <row r="18" spans="1:23" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>10</v>
@@ -4601,28 +4625,28 @@
         <v>6</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="L18" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="M18" s="1"/>
       <c r="N18" s="1"/>
@@ -4632,10 +4656,10 @@
         <v>1</v>
       </c>
       <c r="R18" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="S18" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="T18" s="1"/>
       <c r="U18" s="1"/>
@@ -4644,7 +4668,7 @@
     </row>
     <row r="19" spans="1:23" ht="25" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>49</v>
@@ -4656,26 +4680,26 @@
         <v>6</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F19" s="1"/>
       <c r="G19" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="M19" s="1"/>
       <c r="N19" s="1"/>
@@ -4685,10 +4709,10 @@
         <v>1</v>
       </c>
       <c r="R19" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="S19" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="T19" s="1"/>
       <c r="U19" s="1"/>
@@ -4697,7 +4721,7 @@
     </row>
     <row r="20" spans="1:23" ht="25" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>49</v>
@@ -4709,7 +4733,7 @@
         <v>6</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F20" s="1"/>
       <c r="G20" s="1" t="s">
@@ -4717,16 +4741,16 @@
       </c>
       <c r="H20" s="1"/>
       <c r="I20" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="M20" s="1"/>
       <c r="N20" s="1"/>
@@ -4736,10 +4760,10 @@
         <v>2</v>
       </c>
       <c r="R20" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="S20" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="T20" s="1"/>
       <c r="U20" s="1"/>
@@ -4748,27 +4772,29 @@
     </row>
     <row r="21" spans="1:23" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>49</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>6</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="F21" s="1"/>
+        <v>154</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>231</v>
+      </c>
       <c r="G21" s="1" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="H21" s="1"/>
       <c r="I21" s="1" t="s">
-        <v>232</v>
+        <v>139</v>
       </c>
       <c r="J21" s="1" t="s">
         <v>233</v>
@@ -4784,13 +4810,13 @@
       <c r="O21" s="1"/>
       <c r="P21" s="1"/>
       <c r="Q21" s="1">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="R21" s="1" t="s">
         <v>236</v>
       </c>
       <c r="S21" s="1" t="s">
-        <v>237</v>
+        <v>143</v>
       </c>
       <c r="T21" s="1"/>
       <c r="U21" s="1"/>
@@ -4799,31 +4825,27 @@
     </row>
     <row r="22" spans="1:23" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>49</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>52</v>
+        <v>96</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>6</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>154</v>
-      </c>
+        <v>238</v>
+      </c>
+      <c r="F22" s="1"/>
       <c r="G22" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="H22" s="1" t="s">
+      <c r="H22" s="1"/>
+      <c r="I22" s="1" t="s">
         <v>240</v>
-      </c>
-      <c r="I22" s="1" t="s">
-        <v>138</v>
       </c>
       <c r="J22" s="1" t="s">
         <v>241</v>
@@ -4839,55 +4861,55 @@
       <c r="O22" s="1"/>
       <c r="P22" s="1"/>
       <c r="Q22" s="1">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="R22" s="1" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="S22" s="1" t="s">
-        <v>132</v>
+        <v>245</v>
       </c>
       <c r="T22" s="1"/>
       <c r="U22" s="1"/>
       <c r="V22" s="1"/>
       <c r="W22" s="1"/>
     </row>
-    <row r="23" spans="1:23" ht="25" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:23" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>49</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>65</v>
+        <v>52</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>6</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>124</v>
+        <v>139</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="K23" s="1" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="L23" s="1" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="M23" s="1"/>
       <c r="N23" s="1"/>
@@ -4897,52 +4919,52 @@
         <v>1</v>
       </c>
       <c r="R23" s="1" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="S23" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="T23" s="1"/>
       <c r="U23" s="1"/>
       <c r="V23" s="1"/>
       <c r="W23" s="1"/>
     </row>
-    <row r="24" spans="1:23" ht="37.5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:23" ht="25" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>10</v>
+        <v>49</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>7</v>
+        <v>65</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>6</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>155</v>
+        <v>253</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>156</v>
+        <v>254</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>138</v>
+        <v>125</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>141</v>
+        <v>257</v>
       </c>
       <c r="M24" s="1"/>
       <c r="N24" s="1"/>
@@ -4952,61 +4974,65 @@
         <v>1</v>
       </c>
       <c r="R24" s="1" t="s">
-        <v>155</v>
+        <v>253</v>
       </c>
       <c r="S24" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="T24" s="1"/>
       <c r="U24" s="1"/>
       <c r="V24" s="1"/>
       <c r="W24" s="1"/>
     </row>
-    <row r="25" spans="1:23" ht="25" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:23" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>49</v>
+        <v>10</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>85</v>
+        <v>34</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>7</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>254</v>
-      </c>
-      <c r="F25" s="1"/>
+        <v>154</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>155</v>
+      </c>
       <c r="G25" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="H25" s="1"/>
+        <v>156</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>157</v>
+      </c>
       <c r="I25" s="1" t="s">
-        <v>232</v>
+        <v>139</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="L25" s="1" t="s">
-        <v>257</v>
+        <v>142</v>
       </c>
       <c r="M25" s="1"/>
       <c r="N25" s="1"/>
       <c r="O25" s="1"/>
       <c r="P25" s="1"/>
       <c r="Q25" s="1">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="R25" s="1" t="s">
-        <v>258</v>
+        <v>156</v>
       </c>
       <c r="S25" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="T25" s="1"/>
       <c r="U25" s="1"/>
@@ -5015,95 +5041,91 @@
     </row>
     <row r="26" spans="1:23" ht="25" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>49</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>7</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>121</v>
-      </c>
+        <v>262</v>
+      </c>
+      <c r="F26" s="1"/>
       <c r="G26" s="1" t="s">
-        <v>260</v>
-      </c>
-      <c r="H26" s="1" t="s">
-        <v>261</v>
-      </c>
+        <v>87</v>
+      </c>
+      <c r="H26" s="1"/>
       <c r="I26" s="1" t="s">
-        <v>138</v>
+        <v>240</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="K26" s="1" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="L26" s="1" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="M26" s="1"/>
       <c r="N26" s="1"/>
       <c r="O26" s="1"/>
       <c r="P26" s="1"/>
       <c r="Q26" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="R26" s="1" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="S26" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="T26" s="1"/>
       <c r="U26" s="1"/>
       <c r="V26" s="1"/>
       <c r="W26" s="1"/>
     </row>
-    <row r="27" spans="1:23" ht="37.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:23" ht="25" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>49</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>62</v>
+        <v>91</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>7</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>153</v>
+        <v>121</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>154</v>
+        <v>122</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>210</v>
+        <v>269</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="K27" s="1" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="L27" s="1" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="M27" s="1"/>
       <c r="N27" s="1"/>
@@ -5113,18 +5135,73 @@
         <v>1</v>
       </c>
       <c r="R27" s="1" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="S27" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="T27" s="1"/>
       <c r="U27" s="1"/>
       <c r="V27" s="1"/>
       <c r="W27" s="1"/>
     </row>
+    <row r="28" spans="1:23" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="A28" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="K28" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="L28" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="M28" s="1"/>
+      <c r="N28" s="1"/>
+      <c r="O28" s="1"/>
+      <c r="P28" s="1"/>
+      <c r="Q28" s="1">
+        <v>1</v>
+      </c>
+      <c r="R28" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="S28" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="T28" s="1"/>
+      <c r="U28" s="1"/>
+      <c r="V28" s="1"/>
+      <c r="W28" s="1"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:W27" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A3:W28" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <mergeCells count="2">
     <mergeCell ref="A2:W2"/>
     <mergeCell ref="A1:W1"/>
@@ -5144,7 +5221,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -5154,7 +5231,7 @@
     </row>
     <row r="2" spans="1:6" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
-        <v>271</v>
+        <v>279</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -5170,16 +5247,16 @@
         <v>3</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>273</v>
+        <v>281</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>274</v>
+        <v>282</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>275</v>
+        <v>283</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
@@ -5724,10 +5801,10 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B34" s="1" t="s">
         <v>91</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>90</v>
       </c>
       <c r="C34" s="1">
         <v>1</v>
@@ -5742,10 +5819,10 @@
     </row>
     <row r="35" spans="1:6" ht="25" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B35" s="1" t="s">
         <v>94</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>93</v>
       </c>
       <c r="C35" s="1">
         <v>1</v>
@@ -5760,10 +5837,10 @@
     </row>
     <row r="36" spans="1:6" ht="25" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B36" s="1" t="s">
         <v>96</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>95</v>
       </c>
       <c r="C36" s="1">
         <v>1</v>
@@ -5778,16 +5855,16 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
-        <v>276</v>
+        <v>284</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
       <c r="E37" s="1"/>
       <c r="F37" s="1" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
     </row>
   </sheetData>
@@ -5815,7 +5892,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -5828,7 +5905,7 @@
     </row>
     <row r="2" spans="1:9" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
-        <v>280</v>
+        <v>288</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -5841,45 +5918,45 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>282</v>
+        <v>290</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>283</v>
+        <v>291</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>285</v>
+        <v>293</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>286</v>
+        <v>294</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>287</v>
+        <v>295</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>288</v>
+        <v>296</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>289</v>
+        <v>297</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="25" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>291</v>
+        <v>299</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>292</v>
+        <v>300</v>
       </c>
       <c r="E4" s="1">
         <v>2</v>
@@ -5888,27 +5965,27 @@
         <v>3</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>295</v>
+        <v>303</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>296</v>
+        <v>304</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>297</v>
+        <v>305</v>
       </c>
       <c r="E5" s="1">
         <v>0</v>
@@ -5918,24 +5995,24 @@
       </c>
       <c r="G5" s="1"/>
       <c r="H5" s="1" t="s">
-        <v>298</v>
+        <v>306</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>299</v>
+        <v>307</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="50" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>300</v>
+        <v>308</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>301</v>
+        <v>309</v>
       </c>
       <c r="E6" s="1">
         <v>0</v>
@@ -5945,24 +6022,24 @@
       </c>
       <c r="G6" s="1"/>
       <c r="H6" s="1" t="s">
-        <v>302</v>
+        <v>310</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>303</v>
+        <v>311</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="62.5" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>304</v>
+        <v>312</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>292</v>
+        <v>300</v>
       </c>
       <c r="E7" s="1">
         <v>2</v>
@@ -5971,27 +6048,27 @@
         <v>3</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>305</v>
+        <v>313</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>306</v>
+        <v>314</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>297</v>
+        <v>305</v>
       </c>
       <c r="E8" s="1">
         <v>0</v>
@@ -6001,24 +6078,24 @@
       </c>
       <c r="G8" s="1"/>
       <c r="H8" s="1" t="s">
-        <v>308</v>
+        <v>316</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>309</v>
+        <v>317</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>310</v>
+        <v>318</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>311</v>
+        <v>319</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>301</v>
+        <v>309</v>
       </c>
       <c r="E9" s="1">
         <v>0</v>
@@ -6028,24 +6105,24 @@
       </c>
       <c r="G9" s="1"/>
       <c r="H9" s="1" t="s">
-        <v>312</v>
+        <v>320</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>313</v>
+        <v>321</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>310</v>
+        <v>318</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>314</v>
+        <v>322</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>292</v>
+        <v>300</v>
       </c>
       <c r="E10" s="1">
         <v>2</v>
@@ -6054,27 +6131,27 @@
         <v>3</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>315</v>
+        <v>323</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>316</v>
+        <v>324</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
-        <v>310</v>
+        <v>318</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>317</v>
+        <v>325</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>297</v>
+        <v>305</v>
       </c>
       <c r="E11" s="1">
         <v>0</v>
@@ -6084,24 +6161,24 @@
       </c>
       <c r="G11" s="1"/>
       <c r="H11" s="1" t="s">
-        <v>318</v>
+        <v>326</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>319</v>
+        <v>327</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>321</v>
+        <v>329</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>301</v>
+        <v>309</v>
       </c>
       <c r="E12" s="1">
         <v>0</v>
@@ -6111,24 +6188,24 @@
       </c>
       <c r="G12" s="1"/>
       <c r="H12" s="1" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>323</v>
+        <v>331</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="62.5" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>324</v>
+        <v>332</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>292</v>
+        <v>300</v>
       </c>
       <c r="E13" s="1">
         <v>2</v>
@@ -6137,27 +6214,27 @@
         <v>3</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>326</v>
+        <v>334</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="62.5" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>327</v>
+        <v>335</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>297</v>
+        <v>305</v>
       </c>
       <c r="E14" s="1">
         <v>0</v>
@@ -6167,24 +6244,24 @@
       </c>
       <c r="G14" s="1"/>
       <c r="H14" s="1" t="s">
-        <v>328</v>
+        <v>336</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>326</v>
+        <v>334</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="25" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>329</v>
+        <v>337</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>301</v>
+        <v>309</v>
       </c>
       <c r="E15" s="1">
         <v>0</v>
@@ -6194,24 +6271,24 @@
       </c>
       <c r="G15" s="1"/>
       <c r="H15" s="1" t="s">
-        <v>330</v>
+        <v>338</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>331</v>
+        <v>339</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>332</v>
+        <v>340</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>292</v>
+        <v>300</v>
       </c>
       <c r="E16" s="1">
         <v>2</v>
@@ -6220,27 +6297,27 @@
         <v>3</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>297</v>
+        <v>305</v>
       </c>
       <c r="E17" s="1">
         <v>0</v>
@@ -6250,24 +6327,24 @@
       </c>
       <c r="G17" s="1"/>
       <c r="H17" s="1" t="s">
-        <v>336</v>
+        <v>344</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="25" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>337</v>
+        <v>345</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>301</v>
+        <v>309</v>
       </c>
       <c r="E18" s="1">
         <v>0</v>
@@ -6277,24 +6354,24 @@
       </c>
       <c r="G18" s="1"/>
       <c r="H18" s="1" t="s">
-        <v>338</v>
+        <v>346</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>339</v>
+        <v>347</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>292</v>
+        <v>300</v>
       </c>
       <c r="E19" s="1">
         <v>2</v>
@@ -6303,13 +6380,13 @@
         <v>3</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
     </row>
   </sheetData>
@@ -6335,7 +6412,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -6346,7 +6423,7 @@
     </row>
     <row r="2" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -6363,24 +6440,24 @@
         <v>3</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>347</v>
+        <v>355</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>348</v>
+        <v>356</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>15</v>
@@ -6389,16 +6466,16 @@
         <v>6</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
     </row>
   </sheetData>

</xml_diff>